<commit_message>
Mapping district 8 ship fees
</commit_message>
<xml_diff>
--- a/data/Apr/Data.xlsx
+++ b/data/Apr/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Apr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F482066E-E455-47D4-B642-74C4DC57EED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E36D81-E9C5-4D27-B3F1-4146E2CB238F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-04" sheetId="4" r:id="rId1"/>
@@ -34,6 +34,7 @@
     <sheet name="22-04" sheetId="23" r:id="rId19"/>
     <sheet name="23-04" sheetId="24" r:id="rId20"/>
     <sheet name="24-04" sheetId="25" r:id="rId21"/>
+    <sheet name="25-04" sheetId="26" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7980" uniqueCount="2554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8421" uniqueCount="2674">
   <si>
     <t>THU 4</t>
   </si>
@@ -7303,12 +7304,18 @@
     <t>HD015065</t>
   </si>
   <si>
+    <t>A22/5 phạm thế hiển p3</t>
+  </si>
+  <si>
     <t>Họ Yen</t>
   </si>
   <si>
     <t>HD014983</t>
   </si>
   <si>
+    <t>Toà Central 2, Vinhomes Central Park, số 208 Nguyễn Hữu Cảnh, phường 22</t>
+  </si>
+  <si>
     <t>HD015027</t>
   </si>
   <si>
@@ -7321,6 +7328,9 @@
     <t>HD015189</t>
   </si>
   <si>
+    <t>208 nguyễn hữu cảnh p22 - landmark 3</t>
+  </si>
+  <si>
     <t>HD015129</t>
   </si>
   <si>
@@ -7345,12 +7355,18 @@
     <t>HD014866</t>
   </si>
   <si>
+    <t>132 bến vân đồn p9</t>
+  </si>
+  <si>
     <t>Thơm Thơm</t>
   </si>
   <si>
     <t>HD015104</t>
   </si>
   <si>
+    <t>119 nguyễn văn công p. Hạnh Thông</t>
+  </si>
+  <si>
     <t>Tu Chi Tien</t>
   </si>
   <si>
@@ -7378,6 +7394,9 @@
     <t>HD014563</t>
   </si>
   <si>
+    <t>đường số 104 brillant tower 3 1206 cc đảo kim cương bình trưng tây</t>
+  </si>
+  <si>
     <t>HD015199</t>
   </si>
   <si>
@@ -7390,18 +7409,27 @@
     <t>HD015201</t>
   </si>
   <si>
+    <t>8/14 Trịnh Đình Thảo, Hoà Thạnh</t>
+  </si>
+  <si>
     <t>An Vi</t>
   </si>
   <si>
     <t>HD014867</t>
   </si>
   <si>
+    <t>139/1 dạ nam phường 3</t>
+  </si>
+  <si>
     <t>Hải Dương</t>
   </si>
   <si>
     <t>HD014950</t>
   </si>
   <si>
+    <t>Chung Cư số 1 Tôn Thất Thuyết Lô M1.613</t>
+  </si>
+  <si>
     <t>CUS19950/pe panhaketya</t>
   </si>
   <si>
@@ -7417,21 +7445,33 @@
     <t>HD015022</t>
   </si>
   <si>
+    <t>Sunrise lô D Nguyễn hữa thọ, Xã Phước Kiển</t>
+  </si>
+  <si>
     <t>Nguyen Thi Thu Trang</t>
   </si>
   <si>
     <t>HD014831</t>
   </si>
   <si>
+    <t>13 đường số 3, Khu dân cư phước kiển A, Lê Văn Lương</t>
+  </si>
+  <si>
     <t>bảo bảo fb Phương Phương</t>
   </si>
   <si>
     <t>HD015165</t>
   </si>
   <si>
+    <t>132 bến vân đồn p6</t>
+  </si>
+  <si>
     <t>HD015008</t>
   </si>
   <si>
+    <t>Thý An</t>
+  </si>
+  <si>
     <t>HD014870</t>
   </si>
   <si>
@@ -7447,120 +7487,156 @@
     <t>HD015267</t>
   </si>
   <si>
+    <t>179/13A hoà bình Phường Hiệp Tân</t>
+  </si>
+  <si>
+    <t>Xuân Phát tiktok @xuanphat94</t>
+  </si>
+  <si>
+    <t>HD015085</t>
+  </si>
+  <si>
+    <t>B214bis đường đông hưng thuận 1, phường đông hưng thuận</t>
+  </si>
+  <si>
+    <t>HD015068</t>
+  </si>
+  <si>
+    <t>Phương Quỳnh</t>
+  </si>
+  <si>
+    <t>HD014884</t>
+  </si>
+  <si>
+    <t>6D đường số 2B, Khu Phố 9, Bình Hưng Hòa A</t>
+  </si>
+  <si>
+    <t>HD014965</t>
+  </si>
+  <si>
+    <t>Hà Gia Mẫn</t>
+  </si>
+  <si>
+    <t>HD015024</t>
+  </si>
+  <si>
+    <t>Tk22/26 Nguyễn cảnh chân- cầu ông lãnh</t>
+  </si>
+  <si>
+    <t>Nhớ Nhớ</t>
+  </si>
+  <si>
+    <t>HD015170</t>
+  </si>
+  <si>
+    <t>Sài gòn Mia block A đường 9a khu trung sơn bình hưng</t>
+  </si>
+  <si>
+    <t>HD015010</t>
+  </si>
+  <si>
+    <t>The Sun Avenue S3-Mai Chí thọ</t>
+  </si>
+  <si>
+    <t>HD015082</t>
+  </si>
+  <si>
+    <t>gộp, kh ck shop 865k</t>
+  </si>
+  <si>
+    <t>Nhã Phương</t>
+  </si>
+  <si>
+    <t>HD015029</t>
+  </si>
+  <si>
+    <t>26/2 đường 59 p14</t>
+  </si>
+  <si>
+    <t>Tuyết Nhi</t>
+  </si>
+  <si>
+    <t>HD014894</t>
+  </si>
+  <si>
+    <t>Block d2, chung cư sài gòn riverside (số 4 đào trí, phú thuận)</t>
+  </si>
+  <si>
+    <t>HD014972</t>
+  </si>
+  <si>
+    <t>HD015158</t>
+  </si>
+  <si>
+    <t>Ngọc Phượng</t>
+  </si>
+  <si>
+    <t>HD014928</t>
+  </si>
+  <si>
+    <t>The grand midtown m5 đường số 16 p. Tân Phú</t>
+  </si>
+  <si>
+    <t>HD015089</t>
+  </si>
+  <si>
+    <t>HD014764</t>
+  </si>
+  <si>
+    <t>116a đường số 16 p tân quy</t>
+  </si>
+  <si>
+    <t>Thanh Hà Phạm</t>
+  </si>
+  <si>
+    <t>HD015051</t>
+  </si>
+  <si>
+    <t>29/15 yên thế, p2</t>
+  </si>
+  <si>
+    <t>Yen Nguyen</t>
+  </si>
+  <si>
+    <t>HD015181</t>
+  </si>
+  <si>
+    <t>92g nguyễn hữu cảnh, phường 22</t>
+  </si>
+  <si>
+    <t>fb Trang Nguyen</t>
+  </si>
+  <si>
+    <t>HD015080</t>
+  </si>
+  <si>
+    <t>452/ G33 Phan Văn trị phường 7 Công ty chuyển phát nhanh quốc tế Bm ViNa</t>
+  </si>
+  <si>
+    <t>Trang Nhung</t>
+  </si>
+  <si>
+    <t>HD015083</t>
+  </si>
+  <si>
+    <t>Chung cư Hà độ toà orchid 2</t>
+  </si>
+  <si>
+    <t>Nguyễn Hồng Nga</t>
+  </si>
+  <si>
+    <t>HD014904</t>
+  </si>
+  <si>
+    <t>104/12 Nguyễn Trọng Tuyển, P15</t>
+  </si>
+  <si>
+    <t>HD015264</t>
+  </si>
+  <si>
     <t>179/13A hoà bình</t>
   </si>
   <si>
-    <t>HD015068</t>
-  </si>
-  <si>
-    <t>Phương Quỳnh</t>
-  </si>
-  <si>
-    <t>HD014884</t>
-  </si>
-  <si>
-    <t>6D đường số 2B, Khu Phố 9, Bình Hưng Hòa A</t>
-  </si>
-  <si>
-    <t>HD014965</t>
-  </si>
-  <si>
-    <t>Hà Gia Mẫn</t>
-  </si>
-  <si>
-    <t>HD015024</t>
-  </si>
-  <si>
-    <t>Tk22/26 Nguyễn cảnh chân- cầu ông lãnh</t>
-  </si>
-  <si>
-    <t>Nhớ Nhớ</t>
-  </si>
-  <si>
-    <t>HD015170</t>
-  </si>
-  <si>
-    <t>HD015010</t>
-  </si>
-  <si>
-    <t>The Sun Avenue S3-Mai Chí thọ</t>
-  </si>
-  <si>
-    <t>HD015082</t>
-  </si>
-  <si>
-    <t>Nhã Phương</t>
-  </si>
-  <si>
-    <t>HD015029</t>
-  </si>
-  <si>
-    <t>Tuyết Nhi</t>
-  </si>
-  <si>
-    <t>HD014894</t>
-  </si>
-  <si>
-    <t>HD014972</t>
-  </si>
-  <si>
-    <t>HD015158</t>
-  </si>
-  <si>
-    <t>Ngọc Phượng</t>
-  </si>
-  <si>
-    <t>HD014928</t>
-  </si>
-  <si>
-    <t>HD015089</t>
-  </si>
-  <si>
-    <t>HD014764</t>
-  </si>
-  <si>
-    <t>116a đường số 16 p tân quy</t>
-  </si>
-  <si>
-    <t>Thanh Hà Phạm</t>
-  </si>
-  <si>
-    <t>HD015051</t>
-  </si>
-  <si>
-    <t>29/15 yên thế, p2</t>
-  </si>
-  <si>
-    <t>Yen Nguyen</t>
-  </si>
-  <si>
-    <t>HD015181</t>
-  </si>
-  <si>
-    <t>92g nguyễn hữu cảnh, phường 22</t>
-  </si>
-  <si>
-    <t>HD015080</t>
-  </si>
-  <si>
-    <t>Trang Nhung</t>
-  </si>
-  <si>
-    <t>HD015083</t>
-  </si>
-  <si>
-    <t>Chung cư Hà độ toà orchid 2</t>
-  </si>
-  <si>
-    <t>Nguyễn Hồng Nga</t>
-  </si>
-  <si>
-    <t>HD014904</t>
-  </si>
-  <si>
-    <t>HD015264</t>
-  </si>
-  <si>
     <t>Nguyễn Hương Giang</t>
   </si>
   <si>
@@ -7594,9 +7670,15 @@
     <t>HD014918</t>
   </si>
   <si>
+    <t>mai chí thọ phường an phú Cc lexington block B</t>
+  </si>
+  <si>
     <t>HD015247</t>
   </si>
   <si>
+    <t>82/17/20 đinh tiên hoàng p1</t>
+  </si>
+  <si>
     <t>HD015072</t>
   </si>
   <si>
@@ -7606,43 +7688,31 @@
     <t>HD015100</t>
   </si>
   <si>
+    <t>339 lê văn quới phường bình trị đông A</t>
+  </si>
+  <si>
     <t>Lê Thị Tuyết Trâm</t>
   </si>
   <si>
+    <t>HD014837</t>
+  </si>
+  <si>
+    <t>90/11 dương bá trạc phương rạch ông</t>
+  </si>
+  <si>
     <t>HD015167</t>
   </si>
   <si>
+    <t>chung cư terrace 21 võ trường toản</t>
+  </si>
+  <si>
+    <t>Nguyễn Thùy Vi</t>
+  </si>
+  <si>
     <t>HD015077</t>
   </si>
   <si>
-    <t>208 nguyễn hữu cảnh p22 - landmark 3</t>
-  </si>
-  <si>
-    <t>104/12 Nguyễn Trọng Tuyển, P15</t>
-  </si>
-  <si>
-    <t>Toà Central 2, Vinhomes Central Park, số 208 Nguyễn Hữu Cảnh, phường 22</t>
-  </si>
-  <si>
-    <t>fb Trang Nguyen</t>
-  </si>
-  <si>
-    <t>452/ G33 Phan Văn trị phường 7 Công ty chuyển phát nhanh quốc tế Bm ViNa</t>
-  </si>
-  <si>
-    <t>82/17/20 đinh tiên hoàng p1</t>
-  </si>
-  <si>
-    <t>chung cư terrace 21 võ trường toản</t>
-  </si>
-  <si>
-    <t>119 nguyễn văn công p. Hạnh Thông</t>
-  </si>
-  <si>
-    <t>26/2 đường 59 p14</t>
-  </si>
-  <si>
-    <t>đường số 104 brillant tower 3 1206 cc đảo kim cương bình trưng tây</t>
+    <t>The Tresor,39-39b bến vân đồn</t>
   </si>
   <si>
     <t>MINZZY</t>
@@ -7651,73 +7721,364 @@
     <t>XE TOÀN THẮNG</t>
   </si>
   <si>
-    <t>mai chí thọ phường an phú Cc lexington block B</t>
-  </si>
-  <si>
-    <t>13 đường số 3, Khu dân cư phước kiển A, Lê Văn Lương</t>
-  </si>
-  <si>
-    <t>179/13A hoà bình Phường Hiệp Tân</t>
-  </si>
-  <si>
-    <t>8/14 Trịnh Đình Thảo, Hoà Thạnh</t>
-  </si>
-  <si>
-    <t>Chung Cư số 1 Tôn Thất Thuyết Lô M1.613</t>
-  </si>
-  <si>
-    <t>Xuân Phát tiktok @xuanphat94</t>
-  </si>
-  <si>
-    <t>HD015085</t>
-  </si>
-  <si>
-    <t>B214bis đường đông hưng thuận 1, phường đông hưng thuận</t>
-  </si>
-  <si>
-    <t>132 bến vân đồn p9</t>
-  </si>
-  <si>
-    <t>Thý An</t>
-  </si>
-  <si>
-    <t>Block d2, chung cư sài gòn riverside (số 4 đào trí, phú thuận)</t>
-  </si>
-  <si>
-    <t>The grand midtown m5 đường số 16 p. Tân Phú</t>
-  </si>
-  <si>
-    <t>139/1 dạ nam phường 3</t>
-  </si>
-  <si>
-    <t>Sunrise lô D Nguyễn hữa thọ, Xã Phước Kiển</t>
-  </si>
-  <si>
-    <t>132 bến vân đồn p6</t>
-  </si>
-  <si>
-    <t>Nguyễn Thùy Vi</t>
-  </si>
-  <si>
-    <t>The Tresor,39-39b bến vân đồn</t>
-  </si>
-  <si>
-    <t>339 lê văn quới phường bình trị đông A</t>
-  </si>
-  <si>
-    <t>A22/5 phạm thế hiển p3</t>
-  </si>
-  <si>
-    <t>Sài gòn Mia block A đường 9a khu trung sơn bình hưng</t>
-  </si>
-  <si>
-    <t>HD014837</t>
-  </si>
-  <si>
-    <t>90/11 dương bá trạc phương rạch ông</t>
-  </si>
-  <si>
-    <t>gộp, kh ck shop 865k</t>
+    <t>NGAY 25-4</t>
+  </si>
+  <si>
+    <t>HD015763</t>
+  </si>
+  <si>
+    <t>AT 25-04</t>
+  </si>
+  <si>
+    <t>25-04-2026</t>
+  </si>
+  <si>
+    <t>HD015672</t>
+  </si>
+  <si>
+    <t>Loan Tran</t>
+  </si>
+  <si>
+    <t>HD015680</t>
+  </si>
+  <si>
+    <t>Hằng Nguyễn</t>
+  </si>
+  <si>
+    <t>HD015363</t>
+  </si>
+  <si>
+    <t>HD015600</t>
+  </si>
+  <si>
+    <t>99 đương số 9 KDC bình hưng</t>
+  </si>
+  <si>
+    <t>HD015565</t>
+  </si>
+  <si>
+    <t>Lotus Tram</t>
+  </si>
+  <si>
+    <t>HD015505</t>
+  </si>
+  <si>
+    <t>HD015602</t>
+  </si>
+  <si>
+    <t>thu đuc</t>
+  </si>
+  <si>
+    <t>Nguyễn Hải Phụng</t>
+  </si>
+  <si>
+    <t>HD015693</t>
+  </si>
+  <si>
+    <t>Thuy Trang</t>
+  </si>
+  <si>
+    <t>HD015739</t>
+  </si>
+  <si>
+    <t>A3 Chung cư The Gold View 346 Bến Vân Đồn - P.1</t>
+  </si>
+  <si>
+    <t>HD015528</t>
+  </si>
+  <si>
+    <t>HD015502</t>
+  </si>
+  <si>
+    <t>HĐ015764</t>
+  </si>
+  <si>
+    <t>HD015726</t>
+  </si>
+  <si>
+    <t>HD015418</t>
+  </si>
+  <si>
+    <t>số 13 đường số 9, P13</t>
+  </si>
+  <si>
+    <t>HD015588</t>
+  </si>
+  <si>
+    <t>HD015392</t>
+  </si>
+  <si>
+    <t>MỸ HUYỀN - giữ đơn</t>
+  </si>
+  <si>
+    <t>HD014566</t>
+  </si>
+  <si>
+    <t>HD015574</t>
+  </si>
+  <si>
+    <t>Vũ Duy Tâm - fb Ngoc Nga</t>
+  </si>
+  <si>
+    <t>HD015761</t>
+  </si>
+  <si>
+    <t>HD015334</t>
+  </si>
+  <si>
+    <t>HD015581</t>
+  </si>
+  <si>
+    <t>HD015372</t>
+  </si>
+  <si>
+    <t>Nguyễn Kim Hồng</t>
+  </si>
+  <si>
+    <t>HD015760</t>
+  </si>
+  <si>
+    <t>Minh Trang</t>
+  </si>
+  <si>
+    <t>HD015370</t>
+  </si>
+  <si>
+    <t>Emily Le</t>
+  </si>
+  <si>
+    <t>HD015400</t>
+  </si>
+  <si>
+    <t>281/36 Lê Văn Sỹ P1</t>
+  </si>
+  <si>
+    <t>HD015483</t>
+  </si>
+  <si>
+    <t>Chung cư Hà đô toà orchid 2</t>
+  </si>
+  <si>
+    <t>HD015678</t>
+  </si>
+  <si>
+    <t>Lucie Huỳnh</t>
+  </si>
+  <si>
+    <t>HD015492</t>
+  </si>
+  <si>
+    <t>HD015705</t>
+  </si>
+  <si>
+    <t>Chan Vin</t>
+  </si>
+  <si>
+    <t>HD015702</t>
+  </si>
+  <si>
+    <t>LIBERTY CENTRAL SAIGON RIVERSIDE HOTEL - 17 Ton Duc Thang St</t>
+  </si>
+  <si>
+    <t>HD015571</t>
+  </si>
+  <si>
+    <t>336/43/5e nguyễn văn luôn p12</t>
+  </si>
+  <si>
+    <t>Ngân Hà</t>
+  </si>
+  <si>
+    <t>HD015652</t>
+  </si>
+  <si>
+    <t>Cc dream home 2, lô B, đường 59, p14</t>
+  </si>
+  <si>
+    <t>HD015424</t>
+  </si>
+  <si>
+    <t>Vân Vân</t>
+  </si>
+  <si>
+    <t>HD015567</t>
+  </si>
+  <si>
+    <t>86/36/3 phổ quang, tân sơn hòa</t>
+  </si>
+  <si>
+    <t>HD015527</t>
+  </si>
+  <si>
+    <t>Thuỷ Trúc</t>
+  </si>
+  <si>
+    <t>HD015561</t>
+  </si>
+  <si>
+    <t>Nguyễn Như Ý</t>
+  </si>
+  <si>
+    <t>HD015595</t>
+  </si>
+  <si>
+    <t>HD015736</t>
+  </si>
+  <si>
+    <t>Lê Ngọc Diễm</t>
+  </si>
+  <si>
+    <t>HD015562</t>
+  </si>
+  <si>
+    <t>HD015601</t>
+  </si>
+  <si>
+    <t>980/4b là gốm p8</t>
+  </si>
+  <si>
+    <t>Hoàng Thuý Liên</t>
+  </si>
+  <si>
+    <t>HD015756</t>
+  </si>
+  <si>
+    <t>119 hoàng diệu 2</t>
+  </si>
+  <si>
+    <t>HD015737</t>
+  </si>
+  <si>
+    <t>Dang Thuy Trang</t>
+  </si>
+  <si>
+    <t>Tòa landmark3, vinhome tân cang</t>
+  </si>
+  <si>
+    <t>Nguyễn Hoài An</t>
+  </si>
+  <si>
+    <t>HD015748</t>
+  </si>
+  <si>
+    <t>15 đặng thai mai p7</t>
+  </si>
+  <si>
+    <t>686 Tô Ngọc Vân, P. Tam Bình</t>
+  </si>
+  <si>
+    <t>685 Tân Sơn phường 12</t>
+  </si>
+  <si>
+    <t>Số 3, đường 37,khu dân cư vạn phúc?phường hiệp bình phước</t>
+  </si>
+  <si>
+    <t>29 Tran thi nghĩ p7</t>
+  </si>
+  <si>
+    <t>47 hiệp bình, hiệp bình chánh</t>
+  </si>
+  <si>
+    <t>107/189 Quang Trung P10</t>
+  </si>
+  <si>
+    <t>trâm fb Anne Ng</t>
+  </si>
+  <si>
+    <t>294/22/53 xô viết nghệ tinh,khu phố 21 phường thạnh mỹ tây</t>
+  </si>
+  <si>
+    <t>kh ck shop 685k</t>
+  </si>
+  <si>
+    <t>kh ck shop 730k</t>
+  </si>
+  <si>
+    <t>kh ck shop 1895k</t>
+  </si>
+  <si>
+    <t>tòa B chung cư 9 view phường phước long</t>
+  </si>
+  <si>
+    <t>36 bờ bao tận trắng P. Sơn Kỳ (chung cư celedon cổng diamond brilliant block B2)</t>
+  </si>
+  <si>
+    <t>Chung cư tara. Phường 6. Block B2 tòa khải hoàn</t>
+  </si>
+  <si>
+    <t>TRINH fb Nguyễn --oben</t>
+  </si>
+  <si>
+    <t>Ms Thuyên Tổ Như ari</t>
+  </si>
+  <si>
+    <t>HD015674</t>
+  </si>
+  <si>
+    <t>Chung cư starlight riverside phường bình phú</t>
+  </si>
+  <si>
+    <t>18/10 kdc bảo anh kp40 đường TL26 phường an phú đông</t>
+  </si>
+  <si>
+    <t>28/13 Trần Thiện Chánh p12</t>
+  </si>
+  <si>
+    <t>346 bến vân đồn, P1</t>
+  </si>
+  <si>
+    <t>290 an dương vương phường chợ quán</t>
+  </si>
+  <si>
+    <t>Chung Cư Diamond Brilliant Số 3 Đường N1 phường Tân Sơn Nhì Sảnh B1</t>
+  </si>
+  <si>
+    <t>A22/6 phạm thể hiển p3</t>
+  </si>
+  <si>
+    <t>206/26/10 Lê văn quới, kp4, bình trị đông</t>
+  </si>
+  <si>
+    <t>Eco green sài gòn, đường nguyễn văn linh, phường tân thuận tân Block B</t>
+  </si>
+  <si>
+    <t>Cc cardinal tower B Phường Tân Phú B908</t>
+  </si>
+  <si>
+    <t>NHƯ Ý LÊ</t>
+  </si>
+  <si>
+    <t>Chung cư Callagarden, kdc Greenlife 13C, Đ. Nguyễn Văn Linh, X. Phong Phú</t>
+  </si>
+  <si>
+    <t>YU MY</t>
+  </si>
+  <si>
+    <t>coca kẹ</t>
+  </si>
+  <si>
+    <t>HD015733</t>
+  </si>
+  <si>
+    <t>532/3/93 Kinh Dương Vương. Phường An Lạc</t>
+  </si>
+  <si>
+    <t>Thuy An Dao</t>
+  </si>
+  <si>
+    <t>Sảnh B2 chung cư Emerald phường Sơn Kỳ</t>
+  </si>
+  <si>
+    <t>17 Bùi Thế Mỹ P. Bảy Hiền</t>
+  </si>
+  <si>
+    <t>Thảo Quyên người nhận tên Thuỳ Minh</t>
+  </si>
+  <si>
+    <t>169 Kênh Trung Ương, Ấp 50, Xã Xuân Thới Thượng</t>
+  </si>
+  <si>
+    <t>HD015427</t>
   </si>
 </sst>
 </file>
@@ -31935,10 +32296,12 @@
   <dimension ref="A1:P66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="75.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="11" width="9.140625" customWidth="1"/>
     <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -32048,7 +32411,7 @@
         <v>2414</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>2549</v>
+        <v>2415</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>2238</v>
@@ -32078,13 +32441,13 @@
         <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2415</v>
+        <v>2416</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2416</v>
+        <v>2417</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>2521</v>
+        <v>2418</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>38</v>
@@ -32117,10 +32480,10 @@
         <v>2200</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2417</v>
+        <v>2419</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>116</v>
@@ -32153,13 +32516,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2420</v>
+        <v>2422</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>2519</v>
+        <v>2423</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>38</v>
@@ -32192,7 +32555,7 @@
         <v>1219</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>1221</v>
@@ -32225,10 +32588,10 @@
         <v>18</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>718</v>
@@ -32261,13 +32624,13 @@
         <v>18</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>22</v>
@@ -32300,7 +32663,7 @@
         <v>1429</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>1431</v>
@@ -32336,10 +32699,10 @@
         <v>678</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>2539</v>
+        <v>2432</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>2196</v>
@@ -32369,13 +32732,13 @@
         <v>18</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>2429</v>
+        <v>2433</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>2430</v>
+        <v>2434</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>2526</v>
+        <v>2435</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>46</v>
@@ -32405,13 +32768,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>2431</v>
+        <v>2436</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2432</v>
+        <v>2437</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>2433</v>
+        <v>2438</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>2137</v>
@@ -32444,13 +32807,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>2434</v>
+        <v>2439</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>2435</v>
+        <v>2440</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>2436</v>
+        <v>2441</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>2238</v>
@@ -32483,7 +32846,7 @@
         <v>340</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>2437</v>
+        <v>2442</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>909</v>
@@ -32516,13 +32879,13 @@
         <v>18</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>2438</v>
+        <v>2443</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>2439</v>
+        <v>2444</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>2528</v>
+        <v>2445</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>2133</v>
@@ -32555,7 +32918,7 @@
         <v>894</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>2440</v>
+        <v>2446</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>896</v>
@@ -32591,7 +32954,7 @@
         <v>2398</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>2441</v>
+        <v>2447</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>1866</v>
@@ -32624,13 +32987,13 @@
         <v>18</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>2442</v>
+        <v>2448</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>2443</v>
+        <v>2449</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>2534</v>
+        <v>2450</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>208</v>
@@ -32660,13 +33023,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>2444</v>
+        <v>2451</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>2445</v>
+        <v>2452</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>2543</v>
+        <v>2453</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>2238</v>
@@ -32696,13 +33059,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>2446</v>
+        <v>2454</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>2447</v>
+        <v>2455</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>2535</v>
+        <v>2456</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>2196</v>
@@ -32732,10 +33095,10 @@
         <v>18</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>2448</v>
+        <v>2457</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>2449</v>
+        <v>2458</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>971</v>
@@ -32771,7 +33134,7 @@
         <v>1481</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>2450</v>
+        <v>2459</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>1483</v>
@@ -32804,13 +33167,13 @@
         <v>18</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>2451</v>
+        <v>2460</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>2452</v>
+        <v>2461</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>2544</v>
+        <v>2462</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>111</v>
@@ -32840,13 +33203,13 @@
         <v>18</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>2453</v>
+        <v>2463</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>2454</v>
+        <v>2464</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>2532</v>
+        <v>2465</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>111</v>
@@ -32879,13 +33242,13 @@
         <v>18</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>2455</v>
+        <v>2466</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>2456</v>
+        <v>2467</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>2545</v>
+        <v>2468</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>2196</v>
@@ -32918,7 +33281,7 @@
         <v>1683</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>2457</v>
+        <v>2469</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>1685</v>
@@ -32951,16 +33314,16 @@
         <v>18</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>2540</v>
+        <v>2470</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>2458</v>
+        <v>2471</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>2459</v>
+        <v>2472</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>2460</v>
+        <v>2473</v>
       </c>
       <c r="G29" s="7">
         <v>685</v>
@@ -32987,13 +33350,13 @@
         <v>18</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>2461</v>
+        <v>2474</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>2462</v>
+        <v>2475</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>2533</v>
+        <v>2476</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>208</v>
@@ -33026,13 +33389,13 @@
         <v>18</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>2536</v>
+        <v>2477</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>2537</v>
+        <v>2478</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>2538</v>
+        <v>2479</v>
       </c>
       <c r="F31" s="8">
         <v>12</v>
@@ -33065,7 +33428,7 @@
         <v>161</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>2464</v>
+        <v>2480</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>163</v>
@@ -33098,13 +33461,13 @@
         <v>18</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>2465</v>
+        <v>2481</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>2466</v>
+        <v>2482</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>2467</v>
+        <v>2483</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>22</v>
@@ -33137,7 +33500,7 @@
         <v>65</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>2468</v>
+        <v>2484</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>1203</v>
@@ -33170,13 +33533,13 @@
         <v>18</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>2469</v>
+        <v>2485</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>2470</v>
+        <v>2486</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>2471</v>
+        <v>2487</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>2137</v>
@@ -33188,7 +33551,7 @@
         <v>25</v>
       </c>
       <c r="I35" s="7">
-        <f t="shared" ref="I35:I63" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
         <v>790</v>
       </c>
       <c r="J35" s="7" t="s">
@@ -33206,13 +33569,13 @@
         <v>18</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>2472</v>
+        <v>2488</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>2473</v>
+        <v>2489</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>2550</v>
+        <v>2490</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>143</v>
@@ -33245,10 +33608,10 @@
         <v>1519</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>2474</v>
+        <v>2491</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>2475</v>
+        <v>2492</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>2133</v>
@@ -33278,13 +33641,13 @@
         <v>18</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>2453</v>
+        <v>2463</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>2476</v>
+        <v>2493</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>2532</v>
+        <v>2465</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>111</v>
@@ -33309,7 +33672,7 @@
         <v>2412</v>
       </c>
       <c r="M38" s="7" t="s">
-        <v>2553</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="39" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -33317,13 +33680,13 @@
         <v>18</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>2477</v>
+        <v>2495</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>2478</v>
+        <v>2496</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>2527</v>
+        <v>2497</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>46</v>
@@ -33353,13 +33716,13 @@
         <v>18</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>2479</v>
+        <v>2498</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>2480</v>
+        <v>2499</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>2541</v>
+        <v>2500</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>2187</v>
@@ -33392,7 +33755,7 @@
         <v>593</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>2481</v>
+        <v>2501</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>595</v>
@@ -33428,7 +33791,7 @@
         <v>900</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>2482</v>
+        <v>2502</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>902</v>
@@ -33464,13 +33827,13 @@
         <v>18</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>2483</v>
+        <v>2503</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>2484</v>
+        <v>2504</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>2542</v>
+        <v>2505</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>2187</v>
@@ -33503,7 +33866,7 @@
         <v>271</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>2485</v>
+        <v>2506</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>273</v>
@@ -33539,10 +33902,10 @@
         <v>1411</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>2486</v>
+        <v>2507</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>2487</v>
+        <v>2508</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>2187</v>
@@ -33572,13 +33935,13 @@
         <v>18</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>2488</v>
+        <v>2509</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>2489</v>
+        <v>2510</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>2490</v>
+        <v>2511</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>88</v>
@@ -33608,13 +33971,13 @@
         <v>18</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>2491</v>
+        <v>2512</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>2492</v>
+        <v>2513</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>2493</v>
+        <v>2514</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>38</v>
@@ -33644,13 +34007,13 @@
         <v>18</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>2522</v>
+        <v>2515</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>2494</v>
+        <v>2516</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>2523</v>
+        <v>2517</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>46</v>
@@ -33680,13 +34043,13 @@
         <v>18</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>2495</v>
+        <v>2518</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>2496</v>
+        <v>2519</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>2497</v>
+        <v>2520</v>
       </c>
       <c r="F49" s="8" t="s">
         <v>2242</v>
@@ -33716,13 +34079,13 @@
         <v>18</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>2498</v>
+        <v>2521</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>2499</v>
+        <v>2522</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>81</v>
@@ -33752,13 +34115,13 @@
         <v>18</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>2461</v>
+        <v>2474</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>2500</v>
+        <v>2524</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>2463</v>
+        <v>2525</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>208</v>
@@ -33791,13 +34154,13 @@
         <v>18</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>2501</v>
+        <v>2526</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>2502</v>
+        <v>2527</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>2503</v>
+        <v>2528</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>46</v>
@@ -33827,13 +34190,13 @@
         <v>18</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>2504</v>
+        <v>2529</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>2505</v>
+        <v>2530</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>2506</v>
+        <v>2531</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>2187</v>
@@ -33863,13 +34226,13 @@
         <v>18</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>2507</v>
+        <v>2532</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>2508</v>
+        <v>2533</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>2509</v>
+        <v>2534</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>2137</v>
@@ -33902,7 +34265,7 @@
         <v>1689</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>2510</v>
+        <v>2535</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>1454</v>
@@ -33938,10 +34301,10 @@
         <v>216</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>2511</v>
+        <v>2536</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>2531</v>
+        <v>2537</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>2133</v>
@@ -33974,10 +34337,10 @@
         <v>1599</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>2512</v>
+        <v>2538</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>2524</v>
+        <v>2539</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>38</v>
@@ -34010,7 +34373,7 @@
         <v>1834</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>2513</v>
+        <v>2540</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>1836</v>
@@ -34046,13 +34409,13 @@
         <v>18</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>2514</v>
+        <v>2541</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>2515</v>
+        <v>2542</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>2548</v>
+        <v>2543</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>22</v>
@@ -34082,13 +34445,13 @@
         <v>18</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>2516</v>
+        <v>2544</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>2551</v>
+        <v>2545</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>2552</v>
+        <v>2546</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>2238</v>
@@ -34121,10 +34484,10 @@
         <v>140</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>2517</v>
+        <v>2547</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>2525</v>
+        <v>2548</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>2133</v>
@@ -34154,13 +34517,13 @@
         <v>18</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>2518</v>
+        <v>2550</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>2547</v>
+        <v>2551</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>2196</v>
@@ -34250,7 +34613,7 @@
         <v>40</v>
       </c>
       <c r="I64" s="3">
-        <f t="shared" ref="I64" si="2">G64-H64</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J64" s="3" t="s">
@@ -34271,13 +34634,13 @@
         <v>18</v>
       </c>
       <c r="C65" s="36" t="s">
-        <v>2529</v>
+        <v>2552</v>
       </c>
       <c r="E65" s="36" t="s">
-        <v>2530</v>
+        <v>2553</v>
       </c>
       <c r="I65" s="36">
-        <f t="shared" ref="I65:I66" si="3">G65-H65</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J65" s="36" t="s">
@@ -34313,7 +34676,7 @@
         <v>30</v>
       </c>
       <c r="I66" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>-30</v>
       </c>
       <c r="J66" s="7" t="s">
@@ -34324,6 +34687,1963 @@
       </c>
       <c r="L66" s="7" t="s">
         <v>2412</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
+  <dimension ref="A1:P53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="80" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2554</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>2555</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>752</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G3" s="7">
+        <v>785</v>
+      </c>
+      <c r="H3" s="7">
+        <v>25</v>
+      </c>
+      <c r="I3" s="7">
+        <f t="shared" ref="I3:I35" si="0">G3-H3</f>
+        <v>760</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>2668</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>2558</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>2669</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G4" s="7">
+        <v>775</v>
+      </c>
+      <c r="H4" s="7">
+        <v>25</v>
+      </c>
+      <c r="I4" s="7">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>2559</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>2560</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>2657</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G5" s="7">
+        <v>375</v>
+      </c>
+      <c r="H5" s="7">
+        <v>25</v>
+      </c>
+      <c r="I5" s="7">
+        <f t="shared" si="0"/>
+        <v>350</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>2561</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>2562</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>2635</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G6" s="3">
+        <v>690</v>
+      </c>
+      <c r="H6" s="3">
+        <v>30</v>
+      </c>
+      <c r="I6" s="3">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>2659</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="7">
+        <v>750</v>
+      </c>
+      <c r="H7" s="7">
+        <v>30</v>
+      </c>
+      <c r="I7" s="7">
+        <f t="shared" ref="I7" si="1">G7-H7</f>
+        <v>720</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>2664</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>2563</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>2564</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G8" s="7">
+        <v>775</v>
+      </c>
+      <c r="H8" s="7">
+        <v>35</v>
+      </c>
+      <c r="I8" s="7">
+        <f t="shared" si="0"/>
+        <v>740</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>952</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>2565</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>2638</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>25</v>
+      </c>
+      <c r="I9" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>2643</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>2566</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>2567</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>2637</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G10" s="3">
+        <v>820</v>
+      </c>
+      <c r="H10" s="3">
+        <v>30</v>
+      </c>
+      <c r="I10" s="3">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>2568</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>2653</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>2189</v>
+      </c>
+      <c r="G11" s="7">
+        <v>690</v>
+      </c>
+      <c r="H11" s="7">
+        <v>30</v>
+      </c>
+      <c r="I11" s="7">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>2570</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>2571</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>2647</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G12" s="7">
+        <v>1455</v>
+      </c>
+      <c r="H12" s="7">
+        <v>25</v>
+      </c>
+      <c r="I12" s="7">
+        <f t="shared" si="0"/>
+        <v>1430</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>2573</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>2574</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>2196</v>
+      </c>
+      <c r="G13" s="7">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7">
+        <v>25</v>
+      </c>
+      <c r="I13" s="7">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>2575</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>1781</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G14" s="7">
+        <v>0</v>
+      </c>
+      <c r="H14" s="7">
+        <v>30</v>
+      </c>
+      <c r="I14" s="7">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>2576</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>2646</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>2144</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>30</v>
+      </c>
+      <c r="I15" s="5">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>2639</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G16" s="3">
+        <v>770</v>
+      </c>
+      <c r="H16" s="3">
+        <v>30</v>
+      </c>
+      <c r="I16" s="3">
+        <f t="shared" si="0"/>
+        <v>740</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>2630</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>2578</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>2631</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G17" s="3">
+        <v>550</v>
+      </c>
+      <c r="H17" s="3">
+        <v>20</v>
+      </c>
+      <c r="I17" s="3">
+        <f t="shared" si="0"/>
+        <v>530</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>2662</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>2579</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>2580</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G18" s="7">
+        <v>0</v>
+      </c>
+      <c r="H18" s="7">
+        <v>25</v>
+      </c>
+      <c r="I18" s="7">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>2581</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>1483</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G19" s="7">
+        <v>685</v>
+      </c>
+      <c r="H19" s="7">
+        <v>25</v>
+      </c>
+      <c r="I19" s="7">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>1478</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>2582</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>1480</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>2196</v>
+      </c>
+      <c r="G20" s="7">
+        <v>745</v>
+      </c>
+      <c r="H20" s="7">
+        <v>25</v>
+      </c>
+      <c r="I20" s="7">
+        <f t="shared" si="0"/>
+        <v>720</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>2673</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>1239</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>2183</v>
+      </c>
+      <c r="G21" s="7">
+        <v>0</v>
+      </c>
+      <c r="H21" s="7">
+        <v>25</v>
+      </c>
+      <c r="I21" s="7">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>1689</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>2629</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>1454</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G22" s="3">
+        <v>1455</v>
+      </c>
+      <c r="H22" s="3">
+        <v>25</v>
+      </c>
+      <c r="I22" s="3">
+        <f t="shared" si="0"/>
+        <v>1430</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>2583</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>2584</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>2670</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G23" s="7">
+        <v>25</v>
+      </c>
+      <c r="H23" s="7">
+        <v>25</v>
+      </c>
+      <c r="I23" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>2650</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>2651</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>2189</v>
+      </c>
+      <c r="G24" s="7">
+        <v>0</v>
+      </c>
+      <c r="H24" s="7">
+        <v>30</v>
+      </c>
+      <c r="I24" s="7">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>2586</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>2587</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>2672</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="G25" s="7">
+        <v>1915</v>
+      </c>
+      <c r="H25" s="7">
+        <v>35</v>
+      </c>
+      <c r="I25" s="7">
+        <f t="shared" si="0"/>
+        <v>1880</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>2588</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3">
+        <v>20</v>
+      </c>
+      <c r="I26" s="3">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>2589</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>2655</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>2196</v>
+      </c>
+      <c r="G27" s="7">
+        <v>685</v>
+      </c>
+      <c r="H27" s="7">
+        <v>25</v>
+      </c>
+      <c r="I27" s="7">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>1615</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>2590</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>2661</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G28" s="7">
+        <v>1810</v>
+      </c>
+      <c r="H28" s="7">
+        <v>30</v>
+      </c>
+      <c r="I28" s="7">
+        <f t="shared" si="0"/>
+        <v>1780</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>2591</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>2592</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>2658</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>2238</v>
+      </c>
+      <c r="G29" s="7">
+        <v>690</v>
+      </c>
+      <c r="H29" s="7">
+        <v>30</v>
+      </c>
+      <c r="I29" s="7">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>2593</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>2594</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>2660</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G30" s="7">
+        <v>980</v>
+      </c>
+      <c r="H30" s="7">
+        <v>30</v>
+      </c>
+      <c r="I30" s="7">
+        <f t="shared" si="0"/>
+        <v>950</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>2595</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>2596</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>2597</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G31" s="3">
+        <v>715</v>
+      </c>
+      <c r="H31" s="3">
+        <v>25</v>
+      </c>
+      <c r="I31" s="3">
+        <f t="shared" si="0"/>
+        <v>690</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>2518</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>2598</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>2599</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>2242</v>
+      </c>
+      <c r="G32" s="7">
+        <v>0</v>
+      </c>
+      <c r="H32" s="7">
+        <v>25</v>
+      </c>
+      <c r="I32" s="7">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J32" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K32" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="7" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M32" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>2234</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>2600</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>2236</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G33" s="7">
+        <v>35</v>
+      </c>
+      <c r="H33" s="7">
+        <v>35</v>
+      </c>
+      <c r="I33" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M33" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>2601</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>2602</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>2652</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G34" s="7">
+        <v>815</v>
+      </c>
+      <c r="H34" s="7">
+        <v>25</v>
+      </c>
+      <c r="I34" s="7">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K34" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>2603</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G35" s="7">
+        <v>690</v>
+      </c>
+      <c r="H35" s="7">
+        <v>30</v>
+      </c>
+      <c r="I35" s="7">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>2604</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>2605</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>2606</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G36" s="7">
+        <v>695</v>
+      </c>
+      <c r="H36" s="7">
+        <v>25</v>
+      </c>
+      <c r="I36" s="7">
+        <f t="shared" ref="I36:I52" si="2">G36-H36</f>
+        <v>670</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>2671</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>2607</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>2608</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G37" s="7">
+        <v>815</v>
+      </c>
+      <c r="H37" s="7">
+        <v>25</v>
+      </c>
+      <c r="I37" s="7">
+        <f t="shared" si="2"/>
+        <v>790</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>2609</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>2610</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>2611</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G38" s="3">
+        <v>685</v>
+      </c>
+      <c r="H38" s="3">
+        <v>25</v>
+      </c>
+      <c r="I38" s="3">
+        <f t="shared" si="2"/>
+        <v>660</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>2632</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>2633</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>2634</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G39" s="3">
+        <v>680</v>
+      </c>
+      <c r="H39" s="3">
+        <v>20</v>
+      </c>
+      <c r="I39" s="3">
+        <f t="shared" si="2"/>
+        <v>660</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>2612</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>2640</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G40" s="3">
+        <v>720</v>
+      </c>
+      <c r="H40" s="3">
+        <v>25</v>
+      </c>
+      <c r="I40" s="3">
+        <f t="shared" si="2"/>
+        <v>695</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>2665</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>2666</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>2667</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G41" s="7">
+        <v>690</v>
+      </c>
+      <c r="H41" s="7">
+        <v>30</v>
+      </c>
+      <c r="I41" s="7">
+        <f t="shared" si="2"/>
+        <v>660</v>
+      </c>
+      <c r="J41" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>2613</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>2614</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>2615</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G42" s="3">
+        <v>685</v>
+      </c>
+      <c r="H42" s="3">
+        <v>25</v>
+      </c>
+      <c r="I42" s="3">
+        <f t="shared" si="2"/>
+        <v>660</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L42" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>2649</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>2616</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G43" s="7">
+        <v>815</v>
+      </c>
+      <c r="H43" s="7">
+        <v>25</v>
+      </c>
+      <c r="I43" s="7">
+        <f t="shared" si="2"/>
+        <v>790</v>
+      </c>
+      <c r="J43" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K43" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L43" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>2617</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>2618</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>2663</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G44" s="7">
+        <v>345</v>
+      </c>
+      <c r="H44" s="7">
+        <v>35</v>
+      </c>
+      <c r="I44" s="7">
+        <f t="shared" si="2"/>
+        <v>310</v>
+      </c>
+      <c r="J44" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K44" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L44" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>2619</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>2620</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>2654</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>2242</v>
+      </c>
+      <c r="G45" s="7">
+        <v>875</v>
+      </c>
+      <c r="H45" s="7">
+        <v>25</v>
+      </c>
+      <c r="I45" s="7">
+        <f t="shared" si="2"/>
+        <v>850</v>
+      </c>
+      <c r="J45" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K45" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L45" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>2641</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>2621</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>2642</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G46" s="3">
+        <v>2260</v>
+      </c>
+      <c r="H46" s="3">
+        <v>20</v>
+      </c>
+      <c r="I46" s="3">
+        <f t="shared" si="2"/>
+        <v>2240</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L46" s="3" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M46" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>2622</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>2623</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>2648</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>2238</v>
+      </c>
+      <c r="G47" s="7">
+        <v>690</v>
+      </c>
+      <c r="H47" s="7">
+        <v>30</v>
+      </c>
+      <c r="I47" s="7">
+        <f t="shared" si="2"/>
+        <v>660</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K47" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L47" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>2624</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>2625</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G48" s="7">
+        <v>0</v>
+      </c>
+      <c r="H48" s="7">
+        <v>0</v>
+      </c>
+      <c r="I48" s="7">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J48" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K48" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L48" s="7" t="s">
+        <v>2557</v>
+      </c>
+      <c r="M48" s="7" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>2626</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>2627</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>2656</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>2183</v>
+      </c>
+      <c r="G49" s="7">
+        <v>925</v>
+      </c>
+      <c r="H49" s="7">
+        <v>25</v>
+      </c>
+      <c r="I49" s="7">
+        <f t="shared" si="2"/>
+        <v>900</v>
+      </c>
+      <c r="J49" s="7" t="s">
+        <v>2556</v>
+      </c>
+      <c r="K49" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L49" s="7" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G50" s="3">
+        <v>3955</v>
+      </c>
+      <c r="H50" s="3">
+        <v>35</v>
+      </c>
+      <c r="I50" s="3">
+        <f t="shared" si="2"/>
+        <v>3920</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L50" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>2628</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>2569</v>
+      </c>
+      <c r="G51" s="3">
+        <v>1415</v>
+      </c>
+      <c r="H51" s="3">
+        <v>35</v>
+      </c>
+      <c r="I51" s="3">
+        <f t="shared" si="2"/>
+        <v>1380</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L51" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>2636</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G52" s="3">
+        <v>30</v>
+      </c>
+      <c r="H52" s="3">
+        <v>30</v>
+      </c>
+      <c r="I52" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L52" s="3" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="11" t="s">
+        <v>1689</v>
+      </c>
+      <c r="D53" s="11" t="s">
+        <v>2535</v>
+      </c>
+      <c r="E53" s="11" t="s">
+        <v>1454</v>
+      </c>
+      <c r="F53" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G53" s="11">
+        <v>765</v>
+      </c>
+      <c r="H53" s="11">
+        <v>0</v>
+      </c>
+      <c r="I53" s="11">
+        <f>G53-H53</f>
+        <v>765</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K53" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L53" s="11" t="s">
+        <v>2412</v>
+      </c>
+      <c r="M53" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="N53" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="O53" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="P53" s="11" t="s">
+        <v>431</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update reports in April
</commit_message>
<xml_diff>
--- a/data/Apr/Data.xlsx
+++ b/data/Apr/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Apr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B71B07-6EFE-4FC8-B717-11C035502575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152E4F62-C679-4271-B697-7F243D8C48A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-04" sheetId="4" r:id="rId1"/>
@@ -37,6 +37,7 @@
     <sheet name="25-04" sheetId="26" r:id="rId22"/>
     <sheet name="27-04" sheetId="27" r:id="rId23"/>
     <sheet name="28-04" sheetId="28" r:id="rId24"/>
+    <sheet name="29-04" sheetId="29" r:id="rId25"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9861" uniqueCount="3067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10344" uniqueCount="3213">
   <si>
     <t>THU 4</t>
   </si>
@@ -8965,30 +8966,48 @@
     <t>NGAY 28-4</t>
   </si>
   <si>
+    <t>NGUYỄN MINH DUY</t>
+  </si>
+  <si>
+    <t>90/35 Trần Văn Ơn, Phường Tân Sơn Nhì</t>
+  </si>
+  <si>
+    <t>28-04-2026</t>
+  </si>
+  <si>
+    <t>THƯƠNG 1994</t>
+  </si>
+  <si>
+    <t>Tòa S501, Vinhome grand park, long thạnh mỹ</t>
+  </si>
+  <si>
+    <t>HƯƠNG TRẦN</t>
+  </si>
+  <si>
+    <t>261/26c chu văn an p12</t>
+  </si>
+  <si>
+    <t>Thanh Thanh Tô</t>
+  </si>
+  <si>
+    <t>HD017096</t>
+  </si>
+  <si>
+    <t>2/16 tân lập p8</t>
+  </si>
+  <si>
+    <t>HD016989</t>
+  </si>
+  <si>
     <t>AT 28-04</t>
   </si>
   <si>
-    <t>28-04-2026</t>
-  </si>
-  <si>
-    <t>HƯƠNG TRẦN</t>
-  </si>
-  <si>
-    <t>Thanh Thanh Tô</t>
-  </si>
-  <si>
-    <t>HD017096</t>
-  </si>
-  <si>
-    <t>2/16 tân lập p8</t>
-  </si>
-  <si>
-    <t>HD016989</t>
-  </si>
-  <si>
     <t>Lê Thảo</t>
   </si>
   <si>
+    <t>HD016900</t>
+  </si>
+  <si>
     <t>3 Đặng Dung, P Tân Định</t>
   </si>
   <si>
@@ -8998,6 +9017,15 @@
     <t>HD016775</t>
   </si>
   <si>
+    <t>Landmark 1 vinhome central park p thạnh mỹ tây</t>
+  </si>
+  <si>
+    <t>chi - fb Mi Na</t>
+  </si>
+  <si>
+    <t>HD017060</t>
+  </si>
+  <si>
     <t>1619/29 phạm thế hiển phường 6</t>
   </si>
   <si>
@@ -9013,6 +9041,12 @@
     <t>Thiên Thiên</t>
   </si>
   <si>
+    <t>HD017084</t>
+  </si>
+  <si>
+    <t>20 đường số 6, linh chiểu</t>
+  </si>
+  <si>
     <t>huyền nguyễn</t>
   </si>
   <si>
@@ -9022,6 +9056,9 @@
     <t>Sunwah White House fb Mzzton</t>
   </si>
   <si>
+    <t>HD017045</t>
+  </si>
+  <si>
     <t>90 nguyễn hữu cảnh thạnh mỹ tây</t>
   </si>
   <si>
@@ -9040,6 +9077,9 @@
     <t>HD016907</t>
   </si>
   <si>
+    <t>188 Nguyễn Văn Công, P.3</t>
+  </si>
+  <si>
     <t>HD017134</t>
   </si>
   <si>
@@ -9049,6 +9089,9 @@
     <t>HD016967</t>
   </si>
   <si>
+    <t>22/31/4 đường số 21, Phường 8 (phường Thông Tây Hội mới)</t>
+  </si>
+  <si>
     <t>HD016592</t>
   </si>
   <si>
@@ -9058,6 +9101,9 @@
     <t>HD017135</t>
   </si>
   <si>
+    <t>10/14 âu duong lân p3</t>
+  </si>
+  <si>
     <t>thảo fb Nguyễn Bình Phương Trinh</t>
   </si>
   <si>
@@ -9073,21 +9119,33 @@
     <t>HD016998</t>
   </si>
   <si>
+    <t>536/43/40 âu cơ p. bảy hiền</t>
+  </si>
+  <si>
     <t>HD016824</t>
   </si>
   <si>
+    <t>485 nguyễn đình chiểu</t>
+  </si>
+  <si>
     <t>Khánh Vy Đỗ</t>
   </si>
   <si>
     <t>HD017102</t>
   </si>
   <si>
+    <t>24 đường số 6 - tam phú</t>
+  </si>
+  <si>
     <t>Thảo Susi</t>
   </si>
   <si>
     <t>HD016982</t>
   </si>
   <si>
+    <t>10/16 đường số 8 phường Bình Hưng Hòa</t>
+  </si>
+  <si>
     <t>Lynn Pham</t>
   </si>
   <si>
@@ -9118,6 +9176,9 @@
     <t>HD016850</t>
   </si>
   <si>
+    <t>V6, Sunrise city south tower 23 nguyễn hữu thọ, phường tân hưng</t>
+  </si>
+  <si>
     <t>HD016826</t>
   </si>
   <si>
@@ -9127,24 +9188,51 @@
     <t>HD016990</t>
   </si>
   <si>
+    <t>220/18 Hồ Văn Huê, P.9</t>
+  </si>
+  <si>
     <t>HD017081</t>
   </si>
   <si>
     <t>HD017133</t>
   </si>
   <si>
+    <t>BN182</t>
+  </si>
+  <si>
+    <t>HD017028</t>
+  </si>
+  <si>
     <t>HD016798</t>
   </si>
   <si>
+    <t>Truc Trieu</t>
+  </si>
+  <si>
     <t>HD017106</t>
   </si>
   <si>
+    <t>Số nhà A6, Garden Home Thủ Đức, Đường số 3, QL13, Phường Hiệp Binh Phước</t>
+  </si>
+  <si>
+    <t>người nhận nana - fb Oanh Tống</t>
+  </si>
+  <si>
+    <t>HD016818</t>
+  </si>
+  <si>
     <t>HD016728</t>
   </si>
   <si>
+    <t>Vũ Thùy Dương</t>
+  </si>
+  <si>
     <t>HD016977</t>
   </si>
   <si>
+    <t>96/50/5 đường phạm đăng giảng, bình hưng hòa</t>
+  </si>
+  <si>
     <t>Duyên Huỳnh</t>
   </si>
   <si>
@@ -9169,97 +9257,448 @@
     <t>H0017097</t>
   </si>
   <si>
-    <t>người nhận nana - fb Oanh Tống</t>
-  </si>
-  <si>
-    <t>HD016818</t>
-  </si>
-  <si>
-    <t>24 đường số 6 - tam phú</t>
-  </si>
-  <si>
-    <t>261/26c chu văn an p12</t>
-  </si>
-  <si>
-    <t>22/31/4 đường số 21, Phường 8 (phường Thông Tây Hội mới)</t>
-  </si>
-  <si>
-    <t>HD017084</t>
-  </si>
-  <si>
-    <t>20 đường số 6, linh chiểu</t>
-  </si>
-  <si>
-    <t>HD017028</t>
-  </si>
-  <si>
-    <t>BN182</t>
-  </si>
-  <si>
-    <t>188 Nguyễn Văn Công, P.3</t>
-  </si>
-  <si>
-    <t>90/35 Trần Văn Ơn, Phường Tân Sơn Nhì</t>
-  </si>
-  <si>
-    <t>NGUYỄN MINH DUY</t>
-  </si>
-  <si>
-    <t>HD017045</t>
-  </si>
-  <si>
-    <t>Truc Trieu</t>
-  </si>
-  <si>
-    <t>Số nhà A6, Garden Home Thủ Đức, Đường số 3, QL13, Phường Hiệp Binh Phước</t>
-  </si>
-  <si>
-    <t>536/43/40 âu cơ p. bảy hiền</t>
-  </si>
-  <si>
-    <t>Landmark 1 vinhome central park p thạnh mỹ tây</t>
-  </si>
-  <si>
-    <t>Tòa S501, Vinhome grand park, long thạnh mỹ</t>
-  </si>
-  <si>
-    <t>THƯƠNG 1994</t>
-  </si>
-  <si>
-    <t>485 nguyễn đình chiểu</t>
-  </si>
-  <si>
-    <t>HD016900</t>
-  </si>
-  <si>
-    <t>220/18 Hồ Văn Huê, P.9</t>
-  </si>
-  <si>
-    <t>10/14 âu duong lân p3</t>
-  </si>
-  <si>
-    <t>10/16 đường số 8 phường Bình Hưng Hòa</t>
-  </si>
-  <si>
-    <t>chi - fb Mi Na</t>
-  </si>
-  <si>
-    <t>HD017060</t>
-  </si>
-  <si>
-    <t>V6, Sunrise city south tower 23 nguyễn hữu thọ, phường tân hưng</t>
-  </si>
-  <si>
-    <t>Vũ Thùy Dương</t>
-  </si>
-  <si>
-    <t>96/50/5 đường phạm đăng giảng, bình hưng hòa</t>
-  </si>
-  <si>
     <t>1707 Phạm thế hiển phường bình đông</t>
   </si>
   <si>
     <t>đơn chuyển AT 28-04</t>
+  </si>
+  <si>
+    <t>NGAY 29-4</t>
+  </si>
+  <si>
+    <t>HD017294</t>
+  </si>
+  <si>
+    <t>29-04-2026</t>
+  </si>
+  <si>
+    <t>Phương Như</t>
+  </si>
+  <si>
+    <t>HD017191</t>
+  </si>
+  <si>
+    <t>10 đường số 2 binh thuận tân thuận</t>
+  </si>
+  <si>
+    <t>AT 29-04</t>
+  </si>
+  <si>
+    <t>Như Ý Nguyễn</t>
+  </si>
+  <si>
+    <t>HD017549</t>
+  </si>
+  <si>
+    <t>4 đào trí phường phú thuận</t>
+  </si>
+  <si>
+    <t>Cindy Nguyễn</t>
+  </si>
+  <si>
+    <t>HD017482</t>
+  </si>
+  <si>
+    <t>12/7 đường P - Khu phố Mỹ Tú 2 - P. Tân Hưng</t>
+  </si>
+  <si>
+    <t>Võ Ngọc Đan Thanh</t>
+  </si>
+  <si>
+    <t>HD017534</t>
+  </si>
+  <si>
+    <t>300 Khuông Việt, phường Phú Trung</t>
+  </si>
+  <si>
+    <t>HD017550</t>
+  </si>
+  <si>
+    <t>HD017199</t>
+  </si>
+  <si>
+    <t>Toà Landmark 2</t>
+  </si>
+  <si>
+    <t>HD017210</t>
+  </si>
+  <si>
+    <t>9 tiên lân 17, bà điểm Phòng 306</t>
+  </si>
+  <si>
+    <t>Chanboramey 015738168</t>
+  </si>
+  <si>
+    <t>157 nguyễn du</t>
+  </si>
+  <si>
+    <t>HD017493</t>
+  </si>
+  <si>
+    <t>404 VÕ VĂN TẦN</t>
+  </si>
+  <si>
+    <t>HD017437</t>
+  </si>
+  <si>
+    <t>HD017518</t>
+  </si>
+  <si>
+    <t>212 b/d11 nguyen trai</t>
+  </si>
+  <si>
+    <t>Nguyễn Thu Hoa</t>
+  </si>
+  <si>
+    <t>HD017198</t>
+  </si>
+  <si>
+    <t>190C mai xuân thưởng.p2</t>
+  </si>
+  <si>
+    <t>HD017515</t>
+  </si>
+  <si>
+    <t>Lan Anh Nguyễn</t>
+  </si>
+  <si>
+    <t>HD017489</t>
+  </si>
+  <si>
+    <t>70 đường số 1 KDC nam long</t>
+  </si>
+  <si>
+    <t>smail- huyền trang</t>
+  </si>
+  <si>
+    <t>HD017006</t>
+  </si>
+  <si>
+    <t>124 đường 24b p.bình trị Đông b</t>
+  </si>
+  <si>
+    <t>Minh Nguyễn</t>
+  </si>
+  <si>
+    <t>HD017439</t>
+  </si>
+  <si>
+    <t>Hoa Hoa</t>
+  </si>
+  <si>
+    <t>HD017317</t>
+  </si>
+  <si>
+    <t>Chung cư topaz elite tạ quang bửu p4 Sảnh Dragon 1B</t>
+  </si>
+  <si>
+    <t>HD017442</t>
+  </si>
+  <si>
+    <t>Tran Kim</t>
+  </si>
+  <si>
+    <t>77A Đường số 9, p.Khánh hội</t>
+  </si>
+  <si>
+    <t>Chân Chân</t>
+  </si>
+  <si>
+    <t>HD017536</t>
+  </si>
+  <si>
+    <t>69/15 Võ Thị Liễu, An Phú Đông</t>
+  </si>
+  <si>
+    <t>Bé Ty - fb Anh Lan</t>
+  </si>
+  <si>
+    <t>HD017415</t>
+  </si>
+  <si>
+    <t>532/3/6 Kinh Dương Vương, Phường An Lạc</t>
+  </si>
+  <si>
+    <t>Lucia Nguyễn</t>
+  </si>
+  <si>
+    <t>HD017190</t>
+  </si>
+  <si>
+    <t>Block E eco green nguyễn văn linh</t>
+  </si>
+  <si>
+    <t>Diệu Linh</t>
+  </si>
+  <si>
+    <t>HD017206</t>
+  </si>
+  <si>
+    <t>103 đường số 6, phường Bình Hưng Hòa</t>
+  </si>
+  <si>
+    <t>Minh Hải ( Thanh Phan )</t>
+  </si>
+  <si>
+    <t>HD017443</t>
+  </si>
+  <si>
+    <t>Lê Tố Quyên</t>
+  </si>
+  <si>
+    <t>HD017197</t>
+  </si>
+  <si>
+    <t>149/1 +3 Nơ Trang Long p12</t>
+  </si>
+  <si>
+    <t>HD017179</t>
+  </si>
+  <si>
+    <t>HD017570</t>
+  </si>
+  <si>
+    <t>HD016638</t>
+  </si>
+  <si>
+    <t>Kim Phụng (inst -suicao20_12)</t>
+  </si>
+  <si>
+    <t>HD017491</t>
+  </si>
+  <si>
+    <t>HD017278</t>
+  </si>
+  <si>
+    <t>HD017481</t>
+  </si>
+  <si>
+    <t>Anh Lee</t>
+  </si>
+  <si>
+    <t>HD017305</t>
+  </si>
+  <si>
+    <t>89 lê thị chợ p. phú thuận</t>
+  </si>
+  <si>
+    <t>Thư Mon</t>
+  </si>
+  <si>
+    <t>HD017416</t>
+  </si>
+  <si>
+    <t>Chung cư sài gòn mia, đường 9a, kdc trung sơn, bình hưng</t>
+  </si>
+  <si>
+    <t>HD017205</t>
+  </si>
+  <si>
+    <t>Jemial Vo</t>
+  </si>
+  <si>
+    <t>HD017495</t>
+  </si>
+  <si>
+    <t>Trịnh Thảo Như</t>
+  </si>
+  <si>
+    <t>HD017282</t>
+  </si>
+  <si>
+    <t>Yến Nhi ( chị thảo )</t>
+  </si>
+  <si>
+    <t>HD017513</t>
+  </si>
+  <si>
+    <t>An Nghi</t>
+  </si>
+  <si>
+    <t>HD017459</t>
+  </si>
+  <si>
+    <t>007 Lô B, Đường C6, Cc Tây Thạnh, P. Tây Thạnh</t>
+  </si>
+  <si>
+    <t>HD017005</t>
+  </si>
+  <si>
+    <t>Gia Trân fb Hà Võ</t>
+  </si>
+  <si>
+    <t>HD017164</t>
+  </si>
+  <si>
+    <t>Nhung SaLin</t>
+  </si>
+  <si>
+    <t>HD017163</t>
+  </si>
+  <si>
+    <t>19a Trần Quang diệu p13</t>
+  </si>
+  <si>
+    <t>HD017297</t>
+  </si>
+  <si>
+    <t>hương</t>
+  </si>
+  <si>
+    <t>HD017535</t>
+  </si>
+  <si>
+    <t>97 đường 24A - bình trị đông B</t>
+  </si>
+  <si>
+    <t>HD017173</t>
+  </si>
+  <si>
+    <t>132 bến Vân đồn p6</t>
+  </si>
+  <si>
+    <t>Thiên Trang</t>
+  </si>
+  <si>
+    <t>HD017325</t>
+  </si>
+  <si>
+    <t>221 trần bình trọng p2</t>
+  </si>
+  <si>
+    <t>HD017209</t>
+  </si>
+  <si>
+    <t>HD017479</t>
+  </si>
+  <si>
+    <t>(HLH express): Tổng kho Sài Gòn 9, Lô G2, Đường K1, KCN Cát Lái</t>
+  </si>
+  <si>
+    <t>Cô Ngọc ( gửi Châu)</t>
+  </si>
+  <si>
+    <t>HD017166</t>
+  </si>
+  <si>
+    <t>Hằng</t>
+  </si>
+  <si>
+    <t>HD017480</t>
+  </si>
+  <si>
+    <t>Block A2 Topaz City, số 39 đường Cao Lỗ, P4</t>
+  </si>
+  <si>
+    <t>HD017572</t>
+  </si>
+  <si>
+    <t>SUMO</t>
+  </si>
+  <si>
+    <t>487 le van sy f12</t>
+  </si>
+  <si>
+    <t>438 phan văn trị, p. hạnh thông</t>
+  </si>
+  <si>
+    <t>406/8 Cộng Hoà, phường 13</t>
+  </si>
+  <si>
+    <t>Keo Kimyou</t>
+  </si>
+  <si>
+    <t>Lương Thúy</t>
+  </si>
+  <si>
+    <t>549/3 lê văn thọ</t>
+  </si>
+  <si>
+    <t>128/25 nguyễn lâm p3</t>
+  </si>
+  <si>
+    <t>CHỊ MYMY</t>
+  </si>
+  <si>
+    <t>HD017180</t>
+  </si>
+  <si>
+    <t>175/87/8/4 đường 2 tăng Nhơn Phú b</t>
+  </si>
+  <si>
+    <t>Minh Nguyệt + Lin Xiao + Hàng Aỉ</t>
+  </si>
+  <si>
+    <t>C16-17 lô C1, đường DD5, phường Đông Hưng Thuận</t>
+  </si>
+  <si>
+    <t>7a/5/42 thành thái p14</t>
+  </si>
+  <si>
+    <t>_____lay_____</t>
+  </si>
+  <si>
+    <t>164/22 Vo Thi Sau, D.3</t>
+  </si>
+  <si>
+    <t>thanh (NHẬN HÀNG CHO TRÀ LY)</t>
+  </si>
+  <si>
+    <t>HD016946</t>
+  </si>
+  <si>
+    <t>Loan Đặng</t>
+  </si>
+  <si>
+    <t>45 Lê Anh Xuân Bến Thành</t>
+  </si>
+  <si>
+    <t>39 hồ hảo hớn, P. cô giang</t>
+  </si>
+  <si>
+    <t>HD017537</t>
+  </si>
+  <si>
+    <t>Natalie Nguyen</t>
+  </si>
+  <si>
+    <t>HD017387</t>
+  </si>
+  <si>
+    <t>239/64 Trần Văn Đang, phường 11</t>
+  </si>
+  <si>
+    <t>481/11 Đoàn Văn Bơ, phường Xóm Chiếu</t>
+  </si>
+  <si>
+    <t>5 Lê Quý Đôn phường Võ Thị Sáu</t>
+  </si>
+  <si>
+    <t>Thúy Linh</t>
+  </si>
+  <si>
+    <t>Thuý Stella</t>
+  </si>
+  <si>
+    <t>68/25 trần quang khải p tân định</t>
+  </si>
+  <si>
+    <t>73 hoa sữa phường 7 cầu kiệu</t>
+  </si>
+  <si>
+    <t>HD017543</t>
+  </si>
+  <si>
+    <t>Chí Đinh</t>
+  </si>
+  <si>
+    <t>hẻm 191 cống quỳnh, nhà trọ an house</t>
+  </si>
+  <si>
+    <t>016701721-010535777</t>
+  </si>
+  <si>
+    <t>0898460039</t>
   </si>
 </sst>
 </file>
@@ -9388,7 +9827,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -9427,6 +9866,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -42524,10 +42964,12 @@
   <dimension ref="A1:P48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="39.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="71.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" customWidth="1"/>
+    <col min="7" max="11" width="9.140625" customWidth="1"/>
     <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -42598,10 +43040,10 @@
         <v>18</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>3047</v>
+        <v>2968</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>3046</v>
+        <v>2969</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>208</v>
@@ -42613,7 +43055,7 @@
         <v>50</v>
       </c>
       <c r="I3" s="3">
-        <f t="shared" ref="I3:I47" si="0">G3-H3</f>
+        <f t="shared" ref="I3:I48" si="0">G3-H3</f>
         <v>8980</v>
       </c>
       <c r="J3" s="3" t="s">
@@ -42623,7 +43065,7 @@
         <v>24</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -42659,7 +43101,7 @@
         <v>24</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -42695,7 +43137,7 @@
         <v>24</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -42706,10 +43148,10 @@
         <v>18</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>3054</v>
+        <v>2971</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>3053</v>
+        <v>2972</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>2672</v>
@@ -42731,7 +43173,7 @@
         <v>24</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -42767,7 +43209,7 @@
         <v>24</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -42803,7 +43245,7 @@
         <v>24</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -42839,7 +43281,7 @@
         <v>24</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -42850,10 +43292,10 @@
         <v>18</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>2970</v>
+        <v>2973</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>3039</v>
+        <v>2974</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>38</v>
@@ -42875,7 +43317,7 @@
         <v>24</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -42883,13 +43325,13 @@
         <v>18</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>2971</v>
+        <v>2975</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>2972</v>
+        <v>2976</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>2973</v>
+        <v>2977</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>88</v>
@@ -42911,7 +43353,7 @@
         <v>24</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -42922,7 +43364,7 @@
         <v>47</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>2974</v>
+        <v>2978</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>49</v>
@@ -42941,13 +43383,13 @@
         <v>880</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -42955,13 +43397,13 @@
         <v>18</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>2975</v>
+        <v>2980</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>3056</v>
+        <v>2981</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>2976</v>
+        <v>2982</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>2137</v>
@@ -42983,7 +43425,7 @@
         <v>24</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -42991,13 +43433,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>2977</v>
+        <v>2983</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2978</v>
+        <v>2984</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>3052</v>
+        <v>2985</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>38</v>
@@ -43019,7 +43461,7 @@
         <v>24</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43027,13 +43469,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>3060</v>
+        <v>2986</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>3061</v>
+        <v>2987</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>2979</v>
+        <v>2988</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>2238</v>
@@ -43049,13 +43491,13 @@
         <v>1550</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43063,13 +43505,13 @@
         <v>18</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>2980</v>
+        <v>2989</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>2981</v>
+        <v>2990</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>2982</v>
+        <v>2991</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>143</v>
@@ -43085,13 +43527,13 @@
         <v>790</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="17" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43099,13 +43541,13 @@
         <v>18</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>2983</v>
+        <v>2992</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>3041</v>
+        <v>2993</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>3042</v>
+        <v>2994</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>116</v>
@@ -43127,7 +43569,7 @@
         <v>24</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="18" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43135,10 +43577,10 @@
         <v>18</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>2984</v>
+        <v>2995</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>2985</v>
+        <v>2996</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>698</v>
@@ -43163,7 +43605,7 @@
         <v>24</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
       <c r="M18" s="9" t="s">
         <v>361</v>
@@ -43174,13 +43616,13 @@
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>2986</v>
+        <v>2997</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>3048</v>
+        <v>2998</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>2987</v>
+        <v>2999</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>38</v>
@@ -43202,7 +43644,7 @@
         <v>24</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="20" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43210,13 +43652,13 @@
         <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>2988</v>
+        <v>3000</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>2989</v>
+        <v>3001</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>2990</v>
+        <v>3002</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>88</v>
@@ -43238,7 +43680,7 @@
         <v>24</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="21" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43246,13 +43688,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>2991</v>
+        <v>3003</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>2992</v>
+        <v>3004</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>3045</v>
+        <v>3005</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>46</v>
@@ -43274,7 +43716,7 @@
         <v>24</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>68</v>
@@ -43288,7 +43730,7 @@
         <v>678</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>2993</v>
+        <v>3006</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>680</v>
@@ -43313,7 +43755,7 @@
         <v>24</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="23" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43321,13 +43763,13 @@
         <v>18</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>2994</v>
+        <v>3007</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>2995</v>
+        <v>3008</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>3040</v>
+        <v>3009</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>46</v>
@@ -43349,7 +43791,7 @@
         <v>24</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="24" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43360,7 +43802,7 @@
         <v>2327</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>2996</v>
+        <v>3010</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>2329</v>
@@ -43379,13 +43821,13 @@
         <v>100</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>68</v>
@@ -43396,13 +43838,13 @@
         <v>18</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>2997</v>
+        <v>3011</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>2998</v>
+        <v>3012</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>3058</v>
+        <v>3013</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>2238</v>
@@ -43418,13 +43860,13 @@
         <v>1910</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="26" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43432,13 +43874,13 @@
         <v>18</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>2999</v>
+        <v>3014</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>3000</v>
+        <v>3015</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>3001</v>
+        <v>3016</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>2196</v>
@@ -43460,7 +43902,7 @@
         <v>24</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="27" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43468,13 +43910,13 @@
         <v>18</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>3002</v>
+        <v>3017</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>3003</v>
+        <v>3018</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>3051</v>
+        <v>3019</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>88</v>
@@ -43496,7 +43938,7 @@
         <v>24</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="28" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43507,10 +43949,10 @@
         <v>1734</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>3004</v>
+        <v>3020</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>3055</v>
+        <v>3021</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>2473</v>
@@ -43532,7 +43974,7 @@
         <v>24</v>
       </c>
       <c r="L28" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="29" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43540,13 +43982,13 @@
         <v>18</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>3005</v>
+        <v>3022</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>3006</v>
+        <v>3023</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>3038</v>
+        <v>3024</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>116</v>
@@ -43568,7 +44010,7 @@
         <v>24</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="30" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43576,13 +44018,13 @@
         <v>18</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>3007</v>
+        <v>3025</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>3008</v>
+        <v>3026</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>3059</v>
+        <v>3027</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>22</v>
@@ -43598,13 +44040,13 @@
         <v>1120</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K30" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="31" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43612,13 +44054,13 @@
         <v>18</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>3009</v>
+        <v>3028</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>3010</v>
+        <v>3029</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>3011</v>
+        <v>3030</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>88</v>
@@ -43640,7 +44082,7 @@
         <v>24</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="32" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43648,13 +44090,13 @@
         <v>18</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>3012</v>
+        <v>3031</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>3013</v>
+        <v>3032</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>3014</v>
+        <v>3033</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>2242</v>
@@ -43676,7 +44118,7 @@
         <v>24</v>
       </c>
       <c r="L32" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="33" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43684,10 +44126,10 @@
         <v>18</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>3015</v>
+        <v>3034</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>3016</v>
+        <v>3035</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>2815</v>
@@ -43712,7 +44154,7 @@
         <v>24</v>
       </c>
       <c r="L33" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="34" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43720,13 +44162,13 @@
         <v>18</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>3017</v>
+        <v>3036</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>3018</v>
+        <v>3037</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>3062</v>
+        <v>3038</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>2187</v>
@@ -43742,13 +44184,13 @@
         <v>540</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K34" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="35" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43759,7 +44201,7 @@
         <v>910</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>3019</v>
+        <v>3039</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>912</v>
@@ -43784,7 +44226,7 @@
         <v>24</v>
       </c>
       <c r="L35" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="36" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43792,13 +44234,13 @@
         <v>18</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>3020</v>
+        <v>3040</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>3021</v>
+        <v>3041</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>3057</v>
+        <v>3042</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>81</v>
@@ -43820,7 +44262,7 @@
         <v>24</v>
       </c>
       <c r="L36" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="37" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43831,7 +44273,7 @@
         <v>178</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>3022</v>
+        <v>3043</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>180</v>
@@ -43850,13 +44292,13 @@
         <v>770</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K37" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="38" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -43867,7 +44309,7 @@
         <v>1126</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>3023</v>
+        <v>3044</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>1128</v>
@@ -43886,13 +44328,13 @@
         <v>-30</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K38" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="39" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43900,10 +44342,10 @@
         <v>18</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>3044</v>
+        <v>3045</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>3043</v>
+        <v>3046</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>2008</v>
@@ -43928,7 +44370,7 @@
         <v>24</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="40" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -43939,7 +44381,7 @@
         <v>900</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>3024</v>
+        <v>3047</v>
       </c>
       <c r="E40" s="9" t="s">
         <v>902</v>
@@ -43964,7 +44406,7 @@
         <v>24</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="41" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -43972,10 +44414,10 @@
         <v>18</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>3048</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>3049</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>3025</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>3050</v>
@@ -44000,7 +44442,7 @@
         <v>24</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="42" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -44008,10 +44450,10 @@
         <v>18</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>3036</v>
+        <v>3051</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>3037</v>
+        <v>3052</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>1409</v>
@@ -44036,7 +44478,7 @@
         <v>24</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="43" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -44047,7 +44489,7 @@
         <v>1876</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>3026</v>
+        <v>3053</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>1878</v>
@@ -44072,7 +44514,7 @@
         <v>24</v>
       </c>
       <c r="L43" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="44" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -44080,13 +44522,13 @@
         <v>18</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>3063</v>
+        <v>3054</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>3027</v>
+        <v>3055</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>3064</v>
+        <v>3056</v>
       </c>
       <c r="F44" s="8" t="s">
         <v>22</v>
@@ -44102,13 +44544,13 @@
         <v>-30</v>
       </c>
       <c r="J44" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K44" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L44" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="45" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -44116,13 +44558,13 @@
         <v>18</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>3028</v>
+        <v>3057</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>3029</v>
+        <v>3058</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>3030</v>
+        <v>3059</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>2196</v>
@@ -44144,7 +44586,7 @@
         <v>24</v>
       </c>
       <c r="L45" s="9" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="46" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -44152,13 +44594,13 @@
         <v>18</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>3031</v>
+        <v>3060</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>3032</v>
+        <v>3061</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>3033</v>
+        <v>3062</v>
       </c>
       <c r="F46" s="8" t="s">
         <v>111</v>
@@ -44174,13 +44616,13 @@
         <v>900</v>
       </c>
       <c r="J46" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K46" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L46" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="47" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -44188,10 +44630,10 @@
         <v>18</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>3034</v>
+        <v>3063</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>3035</v>
+        <v>3064</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>3065</v>
@@ -44210,13 +44652,13 @@
         <v>720</v>
       </c>
       <c r="J47" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K47" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L47" s="7" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="48" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -44242,11 +44684,11 @@
         <v>30</v>
       </c>
       <c r="I48" s="7">
-        <f>G48-H48</f>
+        <f t="shared" si="0"/>
         <v>450</v>
       </c>
       <c r="J48" s="7" t="s">
-        <v>2968</v>
+        <v>2979</v>
       </c>
       <c r="K48" s="7" t="s">
         <v>24</v>
@@ -44256,6 +44698,2184 @@
       </c>
       <c r="M48" s="7" t="s">
         <v>3066</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
+  <dimension ref="A1:P60"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" customWidth="1"/>
+    <col min="7" max="11" width="9.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3067</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>1828</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>3068</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>1830</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>2242</v>
+      </c>
+      <c r="G3" s="9">
+        <v>795</v>
+      </c>
+      <c r="H3" s="9">
+        <v>25</v>
+      </c>
+      <c r="I3" s="9">
+        <f t="shared" ref="I3:I34" si="0">G3-H3</f>
+        <v>770</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>3070</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>3071</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>3072</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G4" s="7">
+        <v>720</v>
+      </c>
+      <c r="H4" s="7">
+        <v>30</v>
+      </c>
+      <c r="I4" s="7">
+        <f t="shared" si="0"/>
+        <v>690</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>3074</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>3075</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>3076</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7">
+        <v>30</v>
+      </c>
+      <c r="I5" s="7">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>3077</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>3078</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>3079</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G6" s="7">
+        <v>1980</v>
+      </c>
+      <c r="H6" s="7">
+        <v>30</v>
+      </c>
+      <c r="I6" s="7">
+        <f t="shared" si="0"/>
+        <v>1950</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>3080</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>3081</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>3082</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G7" s="7">
+        <v>945</v>
+      </c>
+      <c r="H7" s="7">
+        <v>25</v>
+      </c>
+      <c r="I7" s="7">
+        <f t="shared" si="0"/>
+        <v>920</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>2151</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>3083</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>971</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7">
+        <v>25</v>
+      </c>
+      <c r="I8" s="7">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>3084</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>3085</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1170</v>
+      </c>
+      <c r="H9" s="3">
+        <v>20</v>
+      </c>
+      <c r="I9" s="3">
+        <f t="shared" si="0"/>
+        <v>1150</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>3086</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>3087</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="G10" s="7">
+        <v>35</v>
+      </c>
+      <c r="H10" s="7">
+        <v>35</v>
+      </c>
+      <c r="I10" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>3069</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>3088</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>3194</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>3089</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9">
+        <v>25</v>
+      </c>
+      <c r="I11" s="9">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>3193</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>3090</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>3091</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>2473</v>
+      </c>
+      <c r="G12" s="9">
+        <v>1635</v>
+      </c>
+      <c r="H12" s="9">
+        <v>25</v>
+      </c>
+      <c r="I12" s="9">
+        <f t="shared" si="0"/>
+        <v>1610</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>3092</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3">
+        <v>20</v>
+      </c>
+      <c r="I13" s="3">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>847</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>3093</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>3094</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G14" s="9">
+        <v>25</v>
+      </c>
+      <c r="H14" s="9">
+        <v>25</v>
+      </c>
+      <c r="I14" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>3095</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>3096</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>3097</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G15" s="7">
+        <v>1805</v>
+      </c>
+      <c r="H15" s="7">
+        <v>25</v>
+      </c>
+      <c r="I15" s="7">
+        <f t="shared" si="0"/>
+        <v>1780</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>894</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>3098</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>896</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" s="9">
+        <v>795</v>
+      </c>
+      <c r="H16" s="9">
+        <v>25</v>
+      </c>
+      <c r="I16" s="9">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>3099</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>3100</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>3101</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G17" s="7">
+        <v>830</v>
+      </c>
+      <c r="H17" s="7">
+        <v>30</v>
+      </c>
+      <c r="I17" s="7">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>3102</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>3103</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>3104</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G18" s="7">
+        <v>890</v>
+      </c>
+      <c r="H18" s="7">
+        <v>30</v>
+      </c>
+      <c r="I18" s="7">
+        <f t="shared" si="0"/>
+        <v>860</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>3105</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>3106</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>3187</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>2144</v>
+      </c>
+      <c r="G19" s="5">
+        <v>820</v>
+      </c>
+      <c r="H19" s="5">
+        <v>30</v>
+      </c>
+      <c r="I19" s="5">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>3107</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>3108</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>3109</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>2238</v>
+      </c>
+      <c r="G20" s="7">
+        <v>910</v>
+      </c>
+      <c r="H20" s="7">
+        <v>30</v>
+      </c>
+      <c r="I20" s="7">
+        <f t="shared" si="0"/>
+        <v>880</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>3110</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>3206</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G21" s="9">
+        <v>815</v>
+      </c>
+      <c r="H21" s="9">
+        <v>25</v>
+      </c>
+      <c r="I21" s="9">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>3111</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>3198</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>3112</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>2196</v>
+      </c>
+      <c r="G22" s="9">
+        <v>1310</v>
+      </c>
+      <c r="H22" s="9">
+        <v>25</v>
+      </c>
+      <c r="I22" s="9">
+        <f t="shared" si="0"/>
+        <v>1285</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K22" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>3069</v>
+      </c>
+      <c r="M22" s="9" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>3113</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>3114</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>3115</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>2189</v>
+      </c>
+      <c r="G23" s="7">
+        <v>20</v>
+      </c>
+      <c r="H23" s="7">
+        <v>20</v>
+      </c>
+      <c r="I23" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>3116</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>3117</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>3118</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="7">
+        <v>1460</v>
+      </c>
+      <c r="H24" s="7">
+        <v>30</v>
+      </c>
+      <c r="I24" s="7">
+        <f t="shared" si="0"/>
+        <v>1430</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>3119</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>3120</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>3121</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G25" s="7">
+        <v>800</v>
+      </c>
+      <c r="H25" s="7">
+        <v>30</v>
+      </c>
+      <c r="I25" s="7">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>3209</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>3208</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>3210</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G26" s="9">
+        <v>465</v>
+      </c>
+      <c r="H26" s="9">
+        <v>25</v>
+      </c>
+      <c r="I26" s="9">
+        <f t="shared" si="0"/>
+        <v>440</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K26" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>3122</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>3123</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>3124</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G27" s="7">
+        <v>950</v>
+      </c>
+      <c r="H27" s="7">
+        <v>30</v>
+      </c>
+      <c r="I27" s="7">
+        <f t="shared" si="0"/>
+        <v>920</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>3125</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>3126</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" s="7">
+        <v>790</v>
+      </c>
+      <c r="H28" s="7">
+        <v>30</v>
+      </c>
+      <c r="I28" s="7">
+        <f t="shared" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>3127</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>3128</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>3129</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1370</v>
+      </c>
+      <c r="H29" s="3">
+        <v>20</v>
+      </c>
+      <c r="I29" s="3">
+        <f t="shared" si="0"/>
+        <v>1350</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>3191</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>3130</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>3192</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G30" s="9">
+        <v>0</v>
+      </c>
+      <c r="H30" s="9">
+        <v>25</v>
+      </c>
+      <c r="I30" s="9">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J30" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K30" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>3195</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>3131</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>3196</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G31" s="9">
+        <v>825</v>
+      </c>
+      <c r="H31" s="9">
+        <v>25</v>
+      </c>
+      <c r="I31" s="9">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K31" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>1452</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>3132</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>1454</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G32" s="3">
+        <v>2090</v>
+      </c>
+      <c r="H32" s="3">
+        <v>25</v>
+      </c>
+      <c r="I32" s="3">
+        <f t="shared" si="0"/>
+        <v>2065</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>3069</v>
+      </c>
+      <c r="M32" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>3133</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>3134</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>3203</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>2473</v>
+      </c>
+      <c r="G33" s="9">
+        <v>0</v>
+      </c>
+      <c r="H33" s="9">
+        <v>25</v>
+      </c>
+      <c r="I33" s="9">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J33" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K33" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>2163</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>3135</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>3197</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>2137</v>
+      </c>
+      <c r="G34" s="9">
+        <v>765</v>
+      </c>
+      <c r="H34" s="9">
+        <v>25</v>
+      </c>
+      <c r="I34" s="9">
+        <f t="shared" si="0"/>
+        <v>740</v>
+      </c>
+      <c r="J34" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K34" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>3136</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G35" s="7">
+        <v>850</v>
+      </c>
+      <c r="H35" s="7">
+        <v>30</v>
+      </c>
+      <c r="I35" s="7">
+        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <v>820</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>3137</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>3138</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>3139</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G36" s="7">
+        <v>1510</v>
+      </c>
+      <c r="H36" s="7">
+        <v>30</v>
+      </c>
+      <c r="I36" s="7">
+        <f t="shared" si="1"/>
+        <v>1480</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>3140</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>3141</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>3142</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G37" s="7">
+        <v>775</v>
+      </c>
+      <c r="H37" s="7">
+        <v>35</v>
+      </c>
+      <c r="I37" s="7">
+        <f t="shared" si="1"/>
+        <v>740</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>3143</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G38" s="7">
+        <v>825</v>
+      </c>
+      <c r="H38" s="7">
+        <v>25</v>
+      </c>
+      <c r="I38" s="7">
+        <f t="shared" si="1"/>
+        <v>800</v>
+      </c>
+      <c r="J38" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K38" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L38" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>3144</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>3145</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>3179</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G39" s="3">
+        <v>945</v>
+      </c>
+      <c r="H39" s="3">
+        <v>25</v>
+      </c>
+      <c r="I39" s="3">
+        <f t="shared" si="1"/>
+        <v>920</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>3146</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>3147</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>3190</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>2242</v>
+      </c>
+      <c r="G40" s="9">
+        <v>775</v>
+      </c>
+      <c r="H40" s="9">
+        <v>25</v>
+      </c>
+      <c r="I40" s="9">
+        <f t="shared" si="1"/>
+        <v>750</v>
+      </c>
+      <c r="J40" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K40" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L40" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>3148</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>3149</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>3180</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G41" s="3">
+        <v>605</v>
+      </c>
+      <c r="H41" s="3">
+        <v>25</v>
+      </c>
+      <c r="I41" s="3">
+        <f t="shared" si="1"/>
+        <v>580</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>3150</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>3151</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>3152</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G42" s="7">
+        <v>1555</v>
+      </c>
+      <c r="H42" s="7">
+        <v>25</v>
+      </c>
+      <c r="I42" s="7">
+        <f t="shared" si="1"/>
+        <v>1530</v>
+      </c>
+      <c r="J42" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K42" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L42" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>2726</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>3153</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>2728</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>2133</v>
+      </c>
+      <c r="G43" s="3">
+        <v>1070</v>
+      </c>
+      <c r="H43" s="3">
+        <v>30</v>
+      </c>
+      <c r="I43" s="3">
+        <f t="shared" si="1"/>
+        <v>1040</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>3154</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>3155</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>3207</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G44" s="9">
+        <v>2460</v>
+      </c>
+      <c r="H44" s="9">
+        <v>20</v>
+      </c>
+      <c r="I44" s="9">
+        <f t="shared" si="1"/>
+        <v>2440</v>
+      </c>
+      <c r="J44" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K44" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>3069</v>
+      </c>
+      <c r="M44" s="9" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>3156</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>3157</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>3158</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>2473</v>
+      </c>
+      <c r="G45" s="9">
+        <v>945</v>
+      </c>
+      <c r="H45" s="9">
+        <v>25</v>
+      </c>
+      <c r="I45" s="9">
+        <f t="shared" si="1"/>
+        <v>920</v>
+      </c>
+      <c r="J45" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K45" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L45" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>1967</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>3159</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>1969</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="G46" s="7">
+        <v>805</v>
+      </c>
+      <c r="H46" s="7">
+        <v>35</v>
+      </c>
+      <c r="I46" s="7">
+        <f t="shared" si="1"/>
+        <v>770</v>
+      </c>
+      <c r="J46" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K46" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L46" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>3160</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>3161</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>3162</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G47" s="7">
+        <v>850</v>
+      </c>
+      <c r="H47" s="7">
+        <v>30</v>
+      </c>
+      <c r="I47" s="7">
+        <f t="shared" si="1"/>
+        <v>820</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K47" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L47" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>3204</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>3163</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>3164</v>
+      </c>
+      <c r="F48" s="10" t="s">
+        <v>2196</v>
+      </c>
+      <c r="G48" s="9">
+        <v>465</v>
+      </c>
+      <c r="H48" s="9">
+        <v>25</v>
+      </c>
+      <c r="I48" s="9">
+        <f t="shared" si="1"/>
+        <v>440</v>
+      </c>
+      <c r="J48" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K48" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L48" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>3165</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>3166</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>3167</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>2183</v>
+      </c>
+      <c r="G49" s="9">
+        <v>825</v>
+      </c>
+      <c r="H49" s="9">
+        <v>25</v>
+      </c>
+      <c r="I49" s="9">
+        <f t="shared" si="1"/>
+        <v>800</v>
+      </c>
+      <c r="J49" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K49" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L49" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>3182</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>3168</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>3183</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G50" s="3">
+        <v>1345</v>
+      </c>
+      <c r="H50" s="3">
+        <v>25</v>
+      </c>
+      <c r="I50" s="3">
+        <f t="shared" si="1"/>
+        <v>1320</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L50" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>3181</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>3169</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>3170</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>2133</v>
+      </c>
+      <c r="G51" s="3">
+        <v>0</v>
+      </c>
+      <c r="H51" s="3">
+        <v>30</v>
+      </c>
+      <c r="I51" s="3">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L51" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>3171</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>3172</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>3202</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>2196</v>
+      </c>
+      <c r="G52" s="9">
+        <v>0</v>
+      </c>
+      <c r="H52" s="9">
+        <v>25</v>
+      </c>
+      <c r="I52" s="9">
+        <f t="shared" si="1"/>
+        <v>-25</v>
+      </c>
+      <c r="J52" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K52" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L52" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>3045</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>3186</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>2189</v>
+      </c>
+      <c r="G53" s="3">
+        <v>0</v>
+      </c>
+      <c r="H53" s="3">
+        <v>30</v>
+      </c>
+      <c r="I53" s="3">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L53" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>3173</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>3174</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>3175</v>
+      </c>
+      <c r="F54" s="8">
+        <v>8</v>
+      </c>
+      <c r="G54" s="7">
+        <v>0</v>
+      </c>
+      <c r="H54" s="7">
+        <v>25</v>
+      </c>
+      <c r="I54" s="7">
+        <f t="shared" si="1"/>
+        <v>-25</v>
+      </c>
+      <c r="J54" s="7" t="s">
+        <v>3073</v>
+      </c>
+      <c r="K54" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L54" s="7" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>3199</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>3200</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>3201</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>2473</v>
+      </c>
+      <c r="G55" s="9">
+        <v>0</v>
+      </c>
+      <c r="H55" s="9">
+        <v>25</v>
+      </c>
+      <c r="I55" s="9">
+        <f t="shared" si="1"/>
+        <v>-25</v>
+      </c>
+      <c r="J55" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K55" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L55" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>3188</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>3176</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>3189</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>2189</v>
+      </c>
+      <c r="G56" s="3">
+        <v>0</v>
+      </c>
+      <c r="H56" s="3">
+        <v>40</v>
+      </c>
+      <c r="I56" s="3">
+        <f t="shared" si="1"/>
+        <v>-40</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L56" s="3" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>3211</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>2282</v>
+      </c>
+      <c r="F57" s="10">
+        <v>5</v>
+      </c>
+      <c r="G57" s="38">
+        <v>0</v>
+      </c>
+      <c r="H57" s="38">
+        <v>25</v>
+      </c>
+      <c r="I57" s="38">
+        <f>G57-H57</f>
+        <v>-25</v>
+      </c>
+      <c r="J57" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="K57" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L57" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>3177</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>3178</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>2473</v>
+      </c>
+      <c r="G58" s="38">
+        <v>6170</v>
+      </c>
+      <c r="H58" s="38">
+        <v>50</v>
+      </c>
+      <c r="I58" s="38">
+        <f t="shared" si="1"/>
+        <v>6120</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K58" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L58" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>3212</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>2282</v>
+      </c>
+      <c r="F59" s="10">
+        <v>5</v>
+      </c>
+      <c r="G59" s="38">
+        <v>0</v>
+      </c>
+      <c r="H59" s="38">
+        <v>25</v>
+      </c>
+      <c r="I59" s="38">
+        <f>G59-H59</f>
+        <v>-25</v>
+      </c>
+      <c r="J59" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="K59" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L59" s="9" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>3185</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>3184</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G60" s="3">
+        <v>25</v>
+      </c>
+      <c r="H60" s="3">
+        <v>25</v>
+      </c>
+      <c r="I60" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J60" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K60" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L60" s="3" t="s">
+        <v>3069</v>
       </c>
     </row>
   </sheetData>

</xml_diff>